<commit_message>
Multi-university build and HTML updates
</commit_message>
<xml_diff>
--- a/Pharma_DS_Course_Overview.xlsx
+++ b/Pharma_DS_Course_Overview.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5F18922-819B-4445-93FC-39CC1825F205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F66950C-3F75-44D3-934C-75841D049CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="10690" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="10690" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDU" sheetId="1" r:id="rId1"/>
-    <sheet name="DS version guide" sheetId="2" r:id="rId2"/>
+    <sheet name="UCPH" sheetId="3" r:id="rId2"/>
+    <sheet name="DS version guide" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SDU!$A$1:$G$28</definedName>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="262">
   <si>
     <t>Course Code</t>
   </si>
@@ -496,6 +497,315 @@
   </si>
   <si>
     <t>https://odin.sdu.dk/sitecore/index.php?a=searchfagbesk&amp;internkode=bafa500&amp;lang=da</t>
+  </si>
+  <si>
+    <t>SFAB20001U</t>
+  </si>
+  <si>
+    <t>Lægemiddeludvikling fra molekyle til menneske</t>
+  </si>
+  <si>
+    <t>Drug Development from Molecule to Man</t>
+  </si>
+  <si>
+    <t>Andrea Heinz</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20001U</t>
+  </si>
+  <si>
+    <t>Development and production of drugs</t>
+  </si>
+  <si>
+    <t>SFAB20002U</t>
+  </si>
+  <si>
+    <t>Kemiske principper</t>
+  </si>
+  <si>
+    <t>Chemical Principles</t>
+  </si>
+  <si>
+    <t>Huiling Mu</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20002U</t>
+  </si>
+  <si>
+    <t>The chemical basis for drugs and drug substances</t>
+  </si>
+  <si>
+    <t>SFAB20004U</t>
+  </si>
+  <si>
+    <t>Cellulær og molekylær biologi</t>
+  </si>
+  <si>
+    <t>Cellular and Molecular Biology</t>
+  </si>
+  <si>
+    <t>Osman Asghar Mirza</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20004U</t>
+  </si>
+  <si>
+    <t>The pharmacological basis for drugs and drug substances</t>
+  </si>
+  <si>
+    <t>SFAB20006U</t>
+  </si>
+  <si>
+    <t>Organisk kemi I</t>
+  </si>
+  <si>
+    <t>Organic Chemistry I – Physicochemical Properties</t>
+  </si>
+  <si>
+    <t>Rasmus Prætorius Clausen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20006U</t>
+  </si>
+  <si>
+    <t>SFAB20023U</t>
+  </si>
+  <si>
+    <t>Farmaceutisk fysisk kemi I</t>
+  </si>
+  <si>
+    <t>Pharmaceutical Physical Chemistry I – Thermodynamics and Equilibria</t>
+  </si>
+  <si>
+    <t>Anan Yaghmur</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20023U</t>
+  </si>
+  <si>
+    <t>SFAB20025U</t>
+  </si>
+  <si>
+    <t>Kvalitetsvurdering af farmaceutiske råvarer</t>
+  </si>
+  <si>
+    <t>Evaluation of Pharmaceutical Substances</t>
+  </si>
+  <si>
+    <t>Jörg P. Kutter</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20025U</t>
+  </si>
+  <si>
+    <t>SFAB20027U</t>
+  </si>
+  <si>
+    <t>Farmaceutisk biologi</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20027U</t>
+  </si>
+  <si>
+    <t>SFAB20029U</t>
+  </si>
+  <si>
+    <t>Organisk kemi II – syntese af lægemiddelstoffer</t>
+  </si>
+  <si>
+    <t>Organic Chemistry II – Synthesis of Drug Compounds</t>
+  </si>
+  <si>
+    <t>Paul Robert Hansen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20029U</t>
+  </si>
+  <si>
+    <t>SFAB20012U</t>
+  </si>
+  <si>
+    <t>Videnskabsteori og samfundsfarmaci</t>
+  </si>
+  <si>
+    <t>Philosophy of Science and Social Pharmacy</t>
+  </si>
+  <si>
+    <t>Ramune Jacobsen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20012U</t>
+  </si>
+  <si>
+    <t>Use of drugs</t>
+  </si>
+  <si>
+    <t>SFAB20013U</t>
+  </si>
+  <si>
+    <t>Basal farmakologi</t>
+  </si>
+  <si>
+    <t>Basic Pharmacology</t>
+  </si>
+  <si>
+    <t>Niels Skotte</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20013U</t>
+  </si>
+  <si>
+    <t>SFAB20017U</t>
+  </si>
+  <si>
+    <t>Farmaceutisk fysisk kemi II</t>
+  </si>
+  <si>
+    <t>Pharmaceutical Physical Chemistry II – Kinetics and Transport Phenomena</t>
+  </si>
+  <si>
+    <t>Jesper Østergaard</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20017U</t>
+  </si>
+  <si>
+    <t>SFAB20015U</t>
+  </si>
+  <si>
+    <t>Biopharmaceuticals – bioorganisk kemi</t>
+  </si>
+  <si>
+    <t>Biopharmaceuticals – Bioorganic Chemistry</t>
+  </si>
+  <si>
+    <t>Henrik Franzyk</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20015U</t>
+  </si>
+  <si>
+    <t>SFAB20033U</t>
+  </si>
+  <si>
+    <t>Samfundsfarmaci – metode og formidling</t>
+  </si>
+  <si>
+    <t>Social Pharmacy – Method and Dissemination</t>
+  </si>
+  <si>
+    <t>Susanne Kaae</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20033U</t>
+  </si>
+  <si>
+    <t>SFAB20035U</t>
+  </si>
+  <si>
+    <t>Farmaceutisk analytisk kemi</t>
+  </si>
+  <si>
+    <t>Pharmaceutical Analytical Chemistry</t>
+  </si>
+  <si>
+    <t>Nickolaj J. Petersen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20035U</t>
+  </si>
+  <si>
+    <t>SFAB20031U</t>
+  </si>
+  <si>
+    <t>Farmaci I – flydende og halvfaste lægemiddelformer</t>
+  </si>
+  <si>
+    <t>Pharmaceutics I – Liquid and Semi-Solid Dosage Forms</t>
+  </si>
+  <si>
+    <t>Hanne Mørck Nielsen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20031U</t>
+  </si>
+  <si>
+    <t>SFAB23001U</t>
+  </si>
+  <si>
+    <t>Organfarmakologi</t>
+  </si>
+  <si>
+    <t>Organ Pharmacology</t>
+  </si>
+  <si>
+    <t>Anders Skov Kristensen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB23001U</t>
+  </si>
+  <si>
+    <t>SFAB20008U</t>
+  </si>
+  <si>
+    <t>Lægemidler fra naturen</t>
+  </si>
+  <si>
+    <t>Drugs from Nature</t>
+  </si>
+  <si>
+    <t>Dan Stærk</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20008U</t>
+  </si>
+  <si>
+    <t>SFAB20010U</t>
+  </si>
+  <si>
+    <t>Farmaci II – faste lægemiddelformer</t>
+  </si>
+  <si>
+    <t>Pharmaceutics II – Solid Dosage Forms</t>
+  </si>
+  <si>
+    <t>Mie Kristensen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20010U</t>
+  </si>
+  <si>
+    <t>SFABIL117U</t>
+  </si>
+  <si>
+    <t>Systemfarmakologi</t>
+  </si>
+  <si>
+    <t>Systems Pharmacology – Signaling Pathways</t>
+  </si>
+  <si>
+    <t>Uffe Kristiansen</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFABIL117U</t>
+  </si>
+  <si>
+    <t>SFAB20019U</t>
+  </si>
+  <si>
+    <t>Farmakoterapi</t>
+  </si>
+  <si>
+    <t>Pharmacotherapy</t>
+  </si>
+  <si>
+    <t>Miriam Kolko</t>
+  </si>
+  <si>
+    <t>https://kurser.ku.dk/course/SFAB20019U</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <t>Version</t>
@@ -526,7 +836,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -581,8 +891,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -647,6 +973,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -716,7 +1066,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -854,10 +1204,46 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
     <dxf>
@@ -2249,6 +2635,721 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F84759-6EDF-44B2-B044-5E0879FECE65}">
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" style="49" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.7109375" style="49" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" style="49" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.7109375" style="49" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" style="49" customWidth="1"/>
+    <col min="8" max="8" width="53" style="49" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="49" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="49" customWidth="1"/>
+    <col min="11" max="11" width="23" style="49" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="49"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="28.5">
+      <c r="A1" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="47" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="47" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="47" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="47" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="47" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="48" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="28.5">
+      <c r="A2" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E2" s="50">
+        <v>1</v>
+      </c>
+      <c r="F2" s="50" t="s">
+        <v>155</v>
+      </c>
+      <c r="G2" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="H2" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="I2" s="50"/>
+      <c r="J2" s="56">
+        <v>1</v>
+      </c>
+      <c r="K2" s="50"/>
+    </row>
+    <row r="3" spans="1:11" ht="28.5">
+      <c r="A3" s="50" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>159</v>
+      </c>
+      <c r="C3" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E3" s="50">
+        <v>1</v>
+      </c>
+      <c r="F3" s="50" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="H3" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I3" s="50"/>
+      <c r="J3" s="57">
+        <v>1</v>
+      </c>
+      <c r="K3" s="50"/>
+    </row>
+    <row r="4" spans="1:11" ht="28.5">
+      <c r="A4" s="50" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E4" s="50">
+        <v>1</v>
+      </c>
+      <c r="F4" s="50" t="s">
+        <v>167</v>
+      </c>
+      <c r="G4" s="50" t="s">
+        <v>168</v>
+      </c>
+      <c r="H4" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I4" s="50"/>
+      <c r="J4" s="57">
+        <v>2</v>
+      </c>
+      <c r="K4" s="50"/>
+    </row>
+    <row r="5" spans="1:11" ht="28.5">
+      <c r="A5" s="50" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="50" t="s">
+        <v>172</v>
+      </c>
+      <c r="D5" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E5" s="50">
+        <v>1</v>
+      </c>
+      <c r="F5" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="G5" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="H5" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I5" s="50"/>
+      <c r="J5" s="57">
+        <v>1</v>
+      </c>
+      <c r="K5" s="50"/>
+    </row>
+    <row r="6" spans="1:11" ht="28.5">
+      <c r="A6" s="50" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" s="50" t="s">
+        <v>176</v>
+      </c>
+      <c r="C6" s="50" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E6" s="50">
+        <v>2</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="I6" s="50"/>
+      <c r="J6" s="57">
+        <v>1</v>
+      </c>
+      <c r="K6" s="50"/>
+    </row>
+    <row r="7" spans="1:11" ht="28.5">
+      <c r="A7" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E7" s="50">
+        <v>2</v>
+      </c>
+      <c r="F7" s="50" t="s">
+        <v>183</v>
+      </c>
+      <c r="G7" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="57">
+        <v>1</v>
+      </c>
+      <c r="K7" s="50"/>
+    </row>
+    <row r="8" spans="1:11" ht="28.5">
+      <c r="A8" s="50" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E8" s="50">
+        <v>2</v>
+      </c>
+      <c r="F8" s="50"/>
+      <c r="G8" s="50" t="s">
+        <v>187</v>
+      </c>
+      <c r="H8" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I8" s="50"/>
+      <c r="J8" s="57">
+        <v>2</v>
+      </c>
+      <c r="K8" s="50"/>
+    </row>
+    <row r="9" spans="1:11" ht="28.5">
+      <c r="A9" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E9" s="50">
+        <v>2</v>
+      </c>
+      <c r="F9" s="50" t="s">
+        <v>191</v>
+      </c>
+      <c r="G9" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="H9" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I9" s="50"/>
+      <c r="J9" s="57">
+        <v>1</v>
+      </c>
+      <c r="K9" s="50"/>
+    </row>
+    <row r="10" spans="1:11" ht="30.75">
+      <c r="A10" s="50" t="s">
+        <v>193</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>194</v>
+      </c>
+      <c r="C10" s="50" t="s">
+        <v>195</v>
+      </c>
+      <c r="D10" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E10" s="50">
+        <v>3</v>
+      </c>
+      <c r="F10" s="50" t="s">
+        <v>196</v>
+      </c>
+      <c r="G10" s="58" t="s">
+        <v>197</v>
+      </c>
+      <c r="H10" s="53" t="s">
+        <v>198</v>
+      </c>
+      <c r="I10" s="50"/>
+      <c r="J10" s="57">
+        <v>1</v>
+      </c>
+      <c r="K10" s="50"/>
+    </row>
+    <row r="11" spans="1:11" ht="30.75">
+      <c r="A11" s="50" t="s">
+        <v>199</v>
+      </c>
+      <c r="B11" s="50" t="s">
+        <v>200</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E11" s="50">
+        <v>3</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="58" t="s">
+        <v>203</v>
+      </c>
+      <c r="H11" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I11" s="50"/>
+      <c r="J11" s="57">
+        <v>2</v>
+      </c>
+      <c r="K11" s="50"/>
+    </row>
+    <row r="12" spans="1:11" ht="30.75">
+      <c r="A12" s="50" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E12" s="50">
+        <v>3</v>
+      </c>
+      <c r="F12" s="50" t="s">
+        <v>207</v>
+      </c>
+      <c r="G12" s="58" t="s">
+        <v>208</v>
+      </c>
+      <c r="H12" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="I12" s="50"/>
+      <c r="J12" s="57">
+        <v>1</v>
+      </c>
+      <c r="K12" s="50"/>
+    </row>
+    <row r="13" spans="1:11" ht="30.75">
+      <c r="A13" s="50" t="s">
+        <v>209</v>
+      </c>
+      <c r="B13" s="50" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="50" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E13" s="50">
+        <v>3</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>212</v>
+      </c>
+      <c r="G13" s="58" t="s">
+        <v>213</v>
+      </c>
+      <c r="H13" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I13" s="50"/>
+      <c r="J13" s="57">
+        <v>1</v>
+      </c>
+      <c r="K13" s="50"/>
+    </row>
+    <row r="14" spans="1:11" ht="30.75">
+      <c r="A14" s="50" t="s">
+        <v>214</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>215</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>216</v>
+      </c>
+      <c r="D14" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E14" s="50">
+        <v>4</v>
+      </c>
+      <c r="F14" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="G14" s="58" t="s">
+        <v>218</v>
+      </c>
+      <c r="H14" s="53" t="s">
+        <v>198</v>
+      </c>
+      <c r="I14" s="50"/>
+      <c r="J14" s="57">
+        <v>1</v>
+      </c>
+      <c r="K14" s="50"/>
+    </row>
+    <row r="15" spans="1:11" ht="30.75">
+      <c r="A15" s="50" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="50" t="s">
+        <v>220</v>
+      </c>
+      <c r="C15" s="50" t="s">
+        <v>221</v>
+      </c>
+      <c r="D15" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E15" s="50">
+        <v>4</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="G15" s="58" t="s">
+        <v>223</v>
+      </c>
+      <c r="H15" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15" s="50"/>
+      <c r="J15" s="57">
+        <v>1</v>
+      </c>
+      <c r="K15" s="50"/>
+    </row>
+    <row r="16" spans="1:11" ht="30.75">
+      <c r="A16" s="50" t="s">
+        <v>224</v>
+      </c>
+      <c r="B16" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="C16" s="50" t="s">
+        <v>226</v>
+      </c>
+      <c r="D16" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E16" s="50">
+        <v>4</v>
+      </c>
+      <c r="F16" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="G16" s="58" t="s">
+        <v>228</v>
+      </c>
+      <c r="H16" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="I16" s="50"/>
+      <c r="J16" s="57">
+        <v>1</v>
+      </c>
+      <c r="K16" s="50"/>
+    </row>
+    <row r="17" spans="1:11" ht="30.75">
+      <c r="A17" s="50" t="s">
+        <v>229</v>
+      </c>
+      <c r="B17" s="50" t="s">
+        <v>230</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>231</v>
+      </c>
+      <c r="D17" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E17" s="50">
+        <v>4</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>232</v>
+      </c>
+      <c r="G17" s="58" t="s">
+        <v>233</v>
+      </c>
+      <c r="H17" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I17" s="50"/>
+      <c r="J17" s="57">
+        <v>1</v>
+      </c>
+      <c r="K17" s="50"/>
+    </row>
+    <row r="18" spans="1:11" ht="28.5">
+      <c r="A18" s="50" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="50" t="s">
+        <v>235</v>
+      </c>
+      <c r="C18" s="50" t="s">
+        <v>236</v>
+      </c>
+      <c r="D18" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E18" s="50">
+        <v>5</v>
+      </c>
+      <c r="F18" s="50" t="s">
+        <v>237</v>
+      </c>
+      <c r="G18" s="50" t="s">
+        <v>238</v>
+      </c>
+      <c r="H18" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="I18" s="50"/>
+      <c r="J18" s="57">
+        <v>1</v>
+      </c>
+      <c r="K18" s="50"/>
+    </row>
+    <row r="19" spans="1:11" ht="30.75">
+      <c r="A19" s="50" t="s">
+        <v>239</v>
+      </c>
+      <c r="B19" s="50" t="s">
+        <v>240</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>241</v>
+      </c>
+      <c r="D19" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E19" s="50">
+        <v>5</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>242</v>
+      </c>
+      <c r="G19" s="58" t="s">
+        <v>243</v>
+      </c>
+      <c r="H19" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="I19" s="50"/>
+      <c r="J19" s="57">
+        <v>1</v>
+      </c>
+      <c r="K19" s="50"/>
+    </row>
+    <row r="20" spans="1:11" ht="30.75">
+      <c r="A20" s="50" t="s">
+        <v>244</v>
+      </c>
+      <c r="B20" s="50" t="s">
+        <v>245</v>
+      </c>
+      <c r="C20" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E20" s="50">
+        <v>5</v>
+      </c>
+      <c r="F20" s="50" t="s">
+        <v>247</v>
+      </c>
+      <c r="G20" s="58" t="s">
+        <v>248</v>
+      </c>
+      <c r="H20" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I20" s="50"/>
+      <c r="J20" s="57">
+        <v>1</v>
+      </c>
+      <c r="K20" s="50"/>
+    </row>
+    <row r="21" spans="1:11" ht="30.75">
+      <c r="A21" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="B21" s="50" t="s">
+        <v>250</v>
+      </c>
+      <c r="C21" s="50" t="s">
+        <v>251</v>
+      </c>
+      <c r="D21" s="50">
+        <v>7.5</v>
+      </c>
+      <c r="E21" s="50">
+        <v>6</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>252</v>
+      </c>
+      <c r="G21" s="58" t="s">
+        <v>253</v>
+      </c>
+      <c r="H21" s="53" t="s">
+        <v>198</v>
+      </c>
+      <c r="I21" s="50"/>
+      <c r="J21" s="57">
+        <v>1</v>
+      </c>
+      <c r="K21" s="50"/>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="50"/>
+      <c r="B22" s="50" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="D22" s="50">
+        <v>15</v>
+      </c>
+      <c r="E22" s="50">
+        <v>6</v>
+      </c>
+      <c r="F22" s="54" t="s">
+        <v>254</v>
+      </c>
+      <c r="G22" s="54" t="s">
+        <v>254</v>
+      </c>
+      <c r="H22" s="50"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="50"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G10" r:id="rId1" xr:uid="{365A484E-6C2B-4A34-B1B6-BA696489541C}"/>
+    <hyperlink ref="G11" r:id="rId2" xr:uid="{593FCE0E-FC11-4319-AA41-AA19488E8DA1}"/>
+    <hyperlink ref="G12" r:id="rId3" xr:uid="{FD7C4E81-194C-47AF-B0F2-EAB99130FEC5}"/>
+    <hyperlink ref="G13" r:id="rId4" xr:uid="{DFB53FC4-2E6C-4947-B60E-DFF6776E1513}"/>
+    <hyperlink ref="G14" r:id="rId5" xr:uid="{849C894D-A75A-47AA-B94E-9A3F1A04793F}"/>
+    <hyperlink ref="G15" r:id="rId6" xr:uid="{D2C2F70E-61F3-461E-8B35-B6D1E5DDEABC}"/>
+    <hyperlink ref="G16" r:id="rId7" xr:uid="{1DE06A8B-3836-487F-B38A-0BEA8BD12E2C}"/>
+    <hyperlink ref="G17" r:id="rId8" xr:uid="{DF9627C9-B486-460D-8DB7-7DC01EB5B5CF}"/>
+    <hyperlink ref="G19" r:id="rId9" xr:uid="{5340029C-171D-4D6B-84F8-322DB73FFDB4}"/>
+    <hyperlink ref="G21" r:id="rId10" xr:uid="{80C30634-6C5B-422D-A8A6-12C1CDE5451F}"/>
+    <hyperlink ref="G20" r:id="rId11" xr:uid="{8C84E52B-5FBD-4018-99BD-769855A47EEB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16E5C0CD-E24B-49F8-83B0-BA99D9C02B58}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2258,10 +3359,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="22" t="s">
-        <v>152</v>
+        <v>255</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>153</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2269,7 +3370,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2277,15 +3378,15 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="45" t="s">
-        <v>156</v>
+        <v>259</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2293,7 +3394,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -2302,15 +3403,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2bc4d9de-87a7-40cc-8fcf-7450ce21fef5">
@@ -2319,6 +3411,15 @@
     <TaxCatchAll xmlns="b6778c44-26f5-4aea-8f0b-e2e010d37707" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2529,11 +3630,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F6CF03-954C-40CE-9E17-9E2B52F08263}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{719C8900-112F-4497-A9C6-71444670DF8F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{719C8900-112F-4497-A9C6-71444670DF8F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92F6CF03-954C-40CE-9E17-9E2B52F08263}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>